<commit_message>
completed eda of building features
</commit_message>
<xml_diff>
--- a/docs/feature_selection_eda.xlsx
+++ b/docs/feature_selection_eda.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HomePC\Desktop\classification_project\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4594AA19-1E32-42DB-B033-6AC58671542E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEFCB562-B502-4627-83BC-6979973F4B2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4C88E5F0-49FA-4653-9B18-637B1C2F945E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="492">
   <si>
     <t>Feature</t>
   </si>
@@ -880,6 +880,636 @@
   </si>
   <si>
     <t>Clearest target relationship within the bureau-request group; retain for baseline and final modeling evaluation</t>
+  </si>
+  <si>
+    <t>apartments_avg</t>
+  </si>
+  <si>
+    <t>Building/Housing</t>
+  </si>
+  <si>
+    <t>Strong decreasing</t>
+  </si>
+  <si>
+    <t>8.72% → 5.80%</t>
+  </si>
+  <si>
+    <t>50.75% missing</t>
+  </si>
+  <si>
+    <t>Strong redundancy with livingarea_avg (0.914), livingapartments_avg (0.944), elevators_avg (0.837)</t>
+  </si>
+  <si>
+    <t>Higher apartment share is associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Clear decreasing bin relationship; useful housing signal despite high missingness</t>
+  </si>
+  <si>
+    <t>basementarea_avg</t>
+  </si>
+  <si>
+    <t>Moderate decreasing</t>
+  </si>
+  <si>
+    <t>Approx. 8.1% → 6.4%</t>
+  </si>
+  <si>
+    <t>58.52% missing</t>
+  </si>
+  <si>
+    <t>Moderate correlation with apartments_avg (0.679) and livingarea_avg (0.693)</t>
+  </si>
+  <si>
+    <t>Higher basement-area share is generally associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Useful directional signal; high missingness should be handled during preprocessing</t>
+  </si>
+  <si>
+    <t>years_beginexpluatation_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.0% → 6.3%</t>
+  </si>
+  <si>
+    <t>48.78% missing</t>
+  </si>
+  <si>
+    <t>Low correlation with most housing features</t>
+  </si>
+  <si>
+    <t>Property exploitation age characteristics show a relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Relatively independent housing signal; retain for modeling review</t>
+  </si>
+  <si>
+    <t>years_build_avg</t>
+  </si>
+  <si>
+    <t>Approx. 7.9% → 6.4%</t>
+  </si>
+  <si>
+    <t>66.50% missing</t>
+  </si>
+  <si>
+    <t>Low/moderate correlation with most housing features</t>
+  </si>
+  <si>
+    <t>Building age characteristics show some relationship with default risk</t>
+  </si>
+  <si>
+    <t>Useful signal but highly missing; final value should be determined by model validation</t>
+  </si>
+  <si>
+    <t>elevators_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.3% → 5.9%</t>
+  </si>
+  <si>
+    <t>53.30% missing; 27.87% zero</t>
+  </si>
+  <si>
+    <t>High correlation with apartments_avg (0.837) and livingarea_avg (0.868)</t>
+  </si>
+  <si>
+    <t>Higher elevator share is associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Strong signal but redundant with property-size features; retain for model comparison</t>
+  </si>
+  <si>
+    <t>floorsmax_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.0% → 6.0%</t>
+  </si>
+  <si>
+    <t>49.76% missing; 0.96% zero</t>
+  </si>
+  <si>
+    <t>Moderate correlation with elevators_avg (0.680); floorsmin_avg (0.742)</t>
+  </si>
+  <si>
+    <t>Building height characteristics show a relationship with default risk</t>
+  </si>
+  <si>
+    <t>Clear directional signal and useful structural information</t>
+  </si>
+  <si>
+    <t>floorsmin_avg</t>
+  </si>
+  <si>
+    <t>Approx. 7.9% → 6.3%</t>
+  </si>
+  <si>
+    <t>67.85% missing; 0.75% zero</t>
+  </si>
+  <si>
+    <t>0.742 with floorsmax_avg</t>
+  </si>
+  <si>
+    <t>Minimum-floor characteristics show some relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Useful signal but highly missing and redundant with floorsmax_avg</t>
+  </si>
+  <si>
+    <t>entrances_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.1% → 6.0%</t>
+  </si>
+  <si>
+    <t>50.35% missing</t>
+  </si>
+  <si>
+    <t>Moderate correlation with basementarea_avg (0.651) and livingarea_avg (0.619)</t>
+  </si>
+  <si>
+    <t>Building entrance characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>Clear directional relationship and meaningful structural information</t>
+  </si>
+  <si>
+    <t>landarea_avg</t>
+  </si>
+  <si>
+    <t>Approx. 7.9% → 6.5%</t>
+  </si>
+  <si>
+    <t>59.38% missing</t>
+  </si>
+  <si>
+    <t>Generally low/moderate correlation with other housing features</t>
+  </si>
+  <si>
+    <t>Larger land-area characteristics are generally associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Potentially useful but weaker signal and high missingness</t>
+  </si>
+  <si>
+    <t>livingarea_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.5% → 5.8%</t>
+  </si>
+  <si>
+    <t>50.19% missing</t>
+  </si>
+  <si>
+    <t>Strong redundancy with apartments_avg (0.914), livingapartments_avg (0.881), elevators_avg (0.868)</t>
+  </si>
+  <si>
+    <t>Higher living-area share is strongly associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Strong target relationship; retain despite redundancy for final model comparison</t>
+  </si>
+  <si>
+    <t>livingapartments_avg</t>
+  </si>
+  <si>
+    <t>Approx. 8.4% → 5.9%</t>
+  </si>
+  <si>
+    <t>68.35% missing</t>
+  </si>
+  <si>
+    <t>Very high correlation with apartments_avg (0.944) and livingarea_avg (0.881)</t>
+  </si>
+  <si>
+    <t>Higher living-apartment share is associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Strong signal but extremely redundant and highly missing; final model will decide</t>
+  </si>
+  <si>
+    <t>nonlivingapartments_avg</t>
+  </si>
+  <si>
+    <t>Weak decreasing</t>
+  </si>
+  <si>
+    <t>Approx. 7.2% → 6.4%</t>
+  </si>
+  <si>
+    <t>69.43% missing</t>
+  </si>
+  <si>
+    <t>Mostly weak correlation with other housing features</t>
+  </si>
+  <si>
+    <t>Non-living apartment characteristics show only a weak relationship with risk</t>
+  </si>
+  <si>
+    <t>Weak signal and very high missingness; low priority for final modeling</t>
+  </si>
+  <si>
+    <t>nonlivingarea_avg</t>
+  </si>
+  <si>
+    <t>Approx. 7.1% → 6.2%</t>
+  </si>
+  <si>
+    <t>55.18% missing; 19.10% zero</t>
+  </si>
+  <si>
+    <t>Non-living area characteristics show a weak relationship with default risk</t>
+  </si>
+  <si>
+    <t>Weak signal; retain temporarily for final model review rather than dropping during EDA</t>
+  </si>
+  <si>
+    <t>commonarea_avg</t>
+  </si>
+  <si>
+    <t>69.87% missing; 2.75% zero</t>
+  </si>
+  <si>
+    <t>Common-area characteristics show some relationship with default risk</t>
+  </si>
+  <si>
+    <t>Potential signal but extremely high missingness; final model validation required</t>
+  </si>
+  <si>
+    <t>apartments_mode</t>
+  </si>
+  <si>
+    <t>Strong decreasing / similar representation</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.15% vs 6.96% non-missing</t>
+  </si>
+  <si>
+    <t>0.973 with apartments_avg; 0.977 with apartments_medi</t>
+  </si>
+  <si>
+    <t>Apartment characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>Highly redundant with other representations; missingness is informative</t>
+  </si>
+  <si>
+    <t>basementarea_mode</t>
+  </si>
+  <si>
+    <t>Moderate decreasing / similar representation</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.91% vs 6.89% non-missing</t>
+  </si>
+  <si>
+    <t>0.973 with basementarea_avg; 0.978 with basementarea_medi</t>
+  </si>
+  <si>
+    <t>Basement-area characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>Highly redundant; high missingness and informative missingness</t>
+  </si>
+  <si>
+    <t>years_beginexpluatation_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.20% vs 6.99% non-missing</t>
+  </si>
+  <si>
+    <t>0.972 with years_beginexpluatation_avg; 0.964 with years_beginexpluatation_medi</t>
+  </si>
+  <si>
+    <t>Property exploitation-age characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>Highly redundant with corresponding representations</t>
+  </si>
+  <si>
+    <t>years_build_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.68% vs 6.87% non-missing</t>
+  </si>
+  <si>
+    <t>0.989 with years_build_avg; 0.989 with years_build_medi</t>
+  </si>
+  <si>
+    <t>Building-age characteristics show some relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Extremely high redundancy and very high missingness</t>
+  </si>
+  <si>
+    <t>commonarea_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.57% vs 6.91% non-missing</t>
+  </si>
+  <si>
+    <t>69.87% missing</t>
+  </si>
+  <si>
+    <t>0.977 with commonarea_avg; 0.980 with commonarea_medi</t>
+  </si>
+  <si>
+    <t>Common-area characteristics show some relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Extremely high missingness and strong redundancy</t>
+  </si>
+  <si>
+    <t>elevators_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.10% vs 6.90% non-missing</t>
+  </si>
+  <si>
+    <t>53.30% missing; 29.10% zero</t>
+  </si>
+  <si>
+    <t>0.979 with elevators_avg; 0.983 with elevators_medi</t>
+  </si>
+  <si>
+    <t>Elevator characteristics are associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Strong redundancy; zero-heavy and high missingness</t>
+  </si>
+  <si>
+    <t>entrances_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.18% vs 6.95% non-missing</t>
+  </si>
+  <si>
+    <t>0.978 with entrances_avg; 0.981 with entrances_medi</t>
+  </si>
+  <si>
+    <t>Highly redundant; missingness is informative</t>
+  </si>
+  <si>
+    <t>floorsmax_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.19% vs 6.97% non-missing</t>
+  </si>
+  <si>
+    <t>49.76% missing; 1.11% zero</t>
+  </si>
+  <si>
+    <t>0.986 with floorsmax_avg; 0.988 with floorsmax_medi</t>
+  </si>
+  <si>
+    <t>Building-height characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>floorsmin_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.63% vs 6.89% non-missing</t>
+  </si>
+  <si>
+    <t>67.85% missing; 0.82% zero</t>
+  </si>
+  <si>
+    <t>0.986 with floorsmin_avg; 0.988 with floorsmin_medi</t>
+  </si>
+  <si>
+    <t>Very high missingness and strong redundancy</t>
+  </si>
+  <si>
+    <t>landarea_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.82% vs 6.98% non-missing</t>
+  </si>
+  <si>
+    <t>59.38% missing; 5.68% zero</t>
+  </si>
+  <si>
+    <t>0.974 with landarea_avg; 0.981 with landarea_medi</t>
+  </si>
+  <si>
+    <t>Land-area characteristics are associated with applicant risk</t>
+  </si>
+  <si>
+    <t>Highly redundant and substantial missingness</t>
+  </si>
+  <si>
+    <t>livingapartments_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.62% vs 6.89% non-missing</t>
+  </si>
+  <si>
+    <t>0.970 with livingapartments_avg; 0.976 with livingapartments_medi</t>
+  </si>
+  <si>
+    <t>Living-apartment characteristics are associated with lower default risk</t>
+  </si>
+  <si>
+    <t>livingarea_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.14% vs 7.00% non-missing</t>
+  </si>
+  <si>
+    <t>0.972 with livingarea_avg; 0.975 with livingarea_medi</t>
+  </si>
+  <si>
+    <t>Higher living-area characteristics are associated with lower default risk</t>
+  </si>
+  <si>
+    <t>nonlivingapartments_mode</t>
+  </si>
+  <si>
+    <t>Weak decreasing / similar representation</t>
+  </si>
+  <si>
+    <t>Missing default rate 8.58% vs 6.91% non-missing</t>
+  </si>
+  <si>
+    <t>69.43% missing; 19.27% zero</t>
+  </si>
+  <si>
+    <t>0.969 with nonlivingapartments_avg; 0.979 with nonlivingapartments_medi</t>
+  </si>
+  <si>
+    <t>Non-living apartment characteristics show limited relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Weak signal, extremely high missingness and strong redundancy</t>
+  </si>
+  <si>
+    <t>nonlivingarea_mode</t>
+  </si>
+  <si>
+    <t>Missing default rate 9.03% vs 6.89% non-missing</t>
+  </si>
+  <si>
+    <t>55.18% missing; 21.83% zero</t>
+  </si>
+  <si>
+    <t>0.966 with nonlivingarea_avg; 0.976 with nonlivingarea_medi</t>
+  </si>
+  <si>
+    <t>Non-living area characteristics show limited relationship with applicant risk</t>
+  </si>
+  <si>
+    <t>Weak signal, substantial missingness and strong redundancy</t>
+  </si>
+  <si>
+    <t>apartments_medi</t>
+  </si>
+  <si>
+    <t>0.995 with apartments_avg; 0.977 with apartments_mode</t>
+  </si>
+  <si>
+    <t>Extremely high redundancy; missingness is informative</t>
+  </si>
+  <si>
+    <t>basementarea_medi</t>
+  </si>
+  <si>
+    <t>0.994 with basementarea_avg; 0.978 with basementarea_mode</t>
+  </si>
+  <si>
+    <t>Extremely high redundancy and high missingness</t>
+  </si>
+  <si>
+    <t>years_beginexpluatation_medi</t>
+  </si>
+  <si>
+    <t>0.994 with years_beginexpluatation_avg; 0.964 with years_beginexpluatation_mode</t>
+  </si>
+  <si>
+    <t>Extremely high redundancy with corresponding representations</t>
+  </si>
+  <si>
+    <t>years_build_medi</t>
+  </si>
+  <si>
+    <t>0.998 with years_build_avg; 0.989 with years_build_mode</t>
+  </si>
+  <si>
+    <t>Near-perfect redundancy and very high missingness</t>
+  </si>
+  <si>
+    <t>commonarea_medi</t>
+  </si>
+  <si>
+    <t>0.996 with commonarea_avg; 0.980 with commonarea_mode</t>
+  </si>
+  <si>
+    <t>Extremely high missingness and near-perfect redundancy</t>
+  </si>
+  <si>
+    <t>elevators_medi</t>
+  </si>
+  <si>
+    <t>53.30% missing; 28.30% zero</t>
+  </si>
+  <si>
+    <t>0.996 with elevators_avg; 0.983 with elevators_mode</t>
+  </si>
+  <si>
+    <t>Near-perfect redundancy; zero-heavy and high missingness</t>
+  </si>
+  <si>
+    <t>entrances_medi</t>
+  </si>
+  <si>
+    <t>0.997 with entrances_avg; 0.981 with entrances_mode</t>
+  </si>
+  <si>
+    <t>Near-perfect redundancy with avg</t>
+  </si>
+  <si>
+    <t>floorsmax_medi</t>
+  </si>
+  <si>
+    <t>49.76% missing; 0.97% zero</t>
+  </si>
+  <si>
+    <t>0.997 with floorsmax_avg; 0.988 with floorsmax_mode</t>
+  </si>
+  <si>
+    <t>floorsmin_medi</t>
+  </si>
+  <si>
+    <t>67.85% missing; 0.76% zero</t>
+  </si>
+  <si>
+    <t>0.997 with floorsmin_avg; 0.988 with floorsmin_mode</t>
+  </si>
+  <si>
+    <t>landarea_medi</t>
+  </si>
+  <si>
+    <t>59.38% missing; 5.18% zero</t>
+  </si>
+  <si>
+    <t>0.992 with landarea_avg; 0.981 with landarea_mode</t>
+  </si>
+  <si>
+    <t>Extremely high redundancy and substantial missingness</t>
+  </si>
+  <si>
+    <t>livingapartments_medi</t>
+  </si>
+  <si>
+    <t>0.994 with livingapartments_avg; 0.976 with livingapartments_mode</t>
+  </si>
+  <si>
+    <t>livingarea_medi</t>
+  </si>
+  <si>
+    <t>0.996 with livingarea_avg; 0.975 with livingarea_mode</t>
+  </si>
+  <si>
+    <t>nonlivingapartments_medi</t>
+  </si>
+  <si>
+    <t>69.43% missing; 18.24% zero</t>
+  </si>
+  <si>
+    <t>0.991 with nonlivingapartments_avg; 0.979 with nonlivingapartments_mode</t>
+  </si>
+  <si>
+    <t>Weak signal, extremely high missingness and near-perfect redundancy</t>
+  </si>
+  <si>
+    <t>nonlivingarea_medi</t>
+  </si>
+  <si>
+    <t>55.18% missing; 19.82% zero</t>
+  </si>
+  <si>
+    <t>0.990 with nonlivingarea_avg; 0.976 with nonlivingarea_mode</t>
+  </si>
+  <si>
+    <t>Weak signal, substantial missingness and near-perfect redundancy</t>
+  </si>
+  <si>
+    <t>totalarea_mode</t>
+  </si>
+  <si>
+    <t>Missing default relationship not separately calculated; binned default rate decreases from 8.85% to 5.56%</t>
+  </si>
+  <si>
+    <t>48.27% missing; 0.19% zero</t>
+  </si>
+  <si>
+    <t>0.899 with livingarea_mode; 0.864 with apartments_mode; 0.834 with livingapartments_mode; 0.821 with elevators_mode</t>
+  </si>
+  <si>
+    <t>Total property area is associated with lower default risk</t>
+  </si>
+  <si>
+    <t>Clear target relationship but highly redundant with several building features; final model validation will determine incremental value</t>
   </si>
 </sst>
 </file>
@@ -1237,7 +1867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1E8CC2-9E90-42FF-9B52-9392EC4342D5}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.26953125" customWidth="1"/>
@@ -3024,7 +3654,1255 @@
         <v>281</v>
       </c>
     </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>282</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C62" t="s">
+        <v>284</v>
+      </c>
+      <c r="D62" t="s">
+        <v>285</v>
+      </c>
+      <c r="E62" t="s">
+        <v>286</v>
+      </c>
+      <c r="F62" t="s">
+        <v>287</v>
+      </c>
+      <c r="G62" t="s">
+        <v>288</v>
+      </c>
+      <c r="H62" t="s">
+        <v>17</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>290</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C63" t="s">
+        <v>291</v>
+      </c>
+      <c r="D63" t="s">
+        <v>292</v>
+      </c>
+      <c r="E63" t="s">
+        <v>293</v>
+      </c>
+      <c r="F63" t="s">
+        <v>294</v>
+      </c>
+      <c r="G63" t="s">
+        <v>295</v>
+      </c>
+      <c r="H63" t="s">
+        <v>17</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>297</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C64" t="s">
+        <v>291</v>
+      </c>
+      <c r="D64" t="s">
+        <v>298</v>
+      </c>
+      <c r="E64" t="s">
+        <v>299</v>
+      </c>
+      <c r="F64" t="s">
+        <v>300</v>
+      </c>
+      <c r="G64" t="s">
+        <v>301</v>
+      </c>
+      <c r="H64" t="s">
+        <v>17</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>303</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C65" t="s">
+        <v>291</v>
+      </c>
+      <c r="D65" t="s">
+        <v>304</v>
+      </c>
+      <c r="E65" t="s">
+        <v>305</v>
+      </c>
+      <c r="F65" t="s">
+        <v>306</v>
+      </c>
+      <c r="G65" t="s">
+        <v>307</v>
+      </c>
+      <c r="H65" t="s">
+        <v>23</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>309</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C66" t="s">
+        <v>284</v>
+      </c>
+      <c r="D66" t="s">
+        <v>310</v>
+      </c>
+      <c r="E66" t="s">
+        <v>311</v>
+      </c>
+      <c r="F66" t="s">
+        <v>312</v>
+      </c>
+      <c r="G66" t="s">
+        <v>313</v>
+      </c>
+      <c r="H66" t="s">
+        <v>23</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>315</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C67" t="s">
+        <v>284</v>
+      </c>
+      <c r="D67" t="s">
+        <v>316</v>
+      </c>
+      <c r="E67" t="s">
+        <v>317</v>
+      </c>
+      <c r="F67" t="s">
+        <v>318</v>
+      </c>
+      <c r="G67" t="s">
+        <v>319</v>
+      </c>
+      <c r="H67" t="s">
+        <v>17</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>321</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C68" t="s">
+        <v>291</v>
+      </c>
+      <c r="D68" t="s">
+        <v>322</v>
+      </c>
+      <c r="E68" t="s">
+        <v>323</v>
+      </c>
+      <c r="F68" t="s">
+        <v>324</v>
+      </c>
+      <c r="G68" t="s">
+        <v>325</v>
+      </c>
+      <c r="H68" t="s">
+        <v>23</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>327</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C69" t="s">
+        <v>284</v>
+      </c>
+      <c r="D69" t="s">
+        <v>328</v>
+      </c>
+      <c r="E69" t="s">
+        <v>329</v>
+      </c>
+      <c r="F69" t="s">
+        <v>330</v>
+      </c>
+      <c r="G69" t="s">
+        <v>331</v>
+      </c>
+      <c r="H69" t="s">
+        <v>17</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>333</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C70" t="s">
+        <v>291</v>
+      </c>
+      <c r="D70" t="s">
+        <v>334</v>
+      </c>
+      <c r="E70" t="s">
+        <v>335</v>
+      </c>
+      <c r="F70" t="s">
+        <v>336</v>
+      </c>
+      <c r="G70" t="s">
+        <v>337</v>
+      </c>
+      <c r="H70" t="s">
+        <v>23</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>339</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C71" t="s">
+        <v>284</v>
+      </c>
+      <c r="D71" t="s">
+        <v>340</v>
+      </c>
+      <c r="E71" t="s">
+        <v>341</v>
+      </c>
+      <c r="F71" t="s">
+        <v>342</v>
+      </c>
+      <c r="G71" t="s">
+        <v>343</v>
+      </c>
+      <c r="H71" t="s">
+        <v>17</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
+        <v>345</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C72" t="s">
+        <v>284</v>
+      </c>
+      <c r="D72" t="s">
+        <v>346</v>
+      </c>
+      <c r="E72" t="s">
+        <v>347</v>
+      </c>
+      <c r="F72" t="s">
+        <v>348</v>
+      </c>
+      <c r="G72" t="s">
+        <v>349</v>
+      </c>
+      <c r="H72" t="s">
+        <v>23</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
+        <v>351</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C73" t="s">
+        <v>352</v>
+      </c>
+      <c r="D73" t="s">
+        <v>353</v>
+      </c>
+      <c r="E73" t="s">
+        <v>354</v>
+      </c>
+      <c r="F73" t="s">
+        <v>355</v>
+      </c>
+      <c r="G73" t="s">
+        <v>356</v>
+      </c>
+      <c r="H73" t="s">
+        <v>23</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
+        <v>358</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C74" t="s">
+        <v>352</v>
+      </c>
+      <c r="D74" t="s">
+        <v>359</v>
+      </c>
+      <c r="E74" t="s">
+        <v>360</v>
+      </c>
+      <c r="F74" t="s">
+        <v>355</v>
+      </c>
+      <c r="G74" t="s">
+        <v>361</v>
+      </c>
+      <c r="H74" t="s">
+        <v>23</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>363</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C75" t="s">
+        <v>291</v>
+      </c>
+      <c r="D75" t="s">
+        <v>298</v>
+      </c>
+      <c r="E75" t="s">
+        <v>364</v>
+      </c>
+      <c r="F75" t="s">
+        <v>336</v>
+      </c>
+      <c r="G75" t="s">
+        <v>365</v>
+      </c>
+      <c r="H75" t="s">
+        <v>23</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
+        <v>367</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C76" t="s">
+        <v>368</v>
+      </c>
+      <c r="D76" t="s">
+        <v>369</v>
+      </c>
+      <c r="E76" t="s">
+        <v>286</v>
+      </c>
+      <c r="F76" t="s">
+        <v>370</v>
+      </c>
+      <c r="G76" t="s">
+        <v>371</v>
+      </c>
+      <c r="H76" t="s">
+        <v>23</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>373</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C77" t="s">
+        <v>374</v>
+      </c>
+      <c r="D77" t="s">
+        <v>375</v>
+      </c>
+      <c r="E77" t="s">
+        <v>293</v>
+      </c>
+      <c r="F77" t="s">
+        <v>376</v>
+      </c>
+      <c r="G77" t="s">
+        <v>377</v>
+      </c>
+      <c r="H77" t="s">
+        <v>23</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>379</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C78" t="s">
+        <v>374</v>
+      </c>
+      <c r="D78" t="s">
+        <v>380</v>
+      </c>
+      <c r="E78" t="s">
+        <v>299</v>
+      </c>
+      <c r="F78" t="s">
+        <v>381</v>
+      </c>
+      <c r="G78" t="s">
+        <v>382</v>
+      </c>
+      <c r="H78" t="s">
+        <v>23</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>384</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C79" t="s">
+        <v>374</v>
+      </c>
+      <c r="D79" t="s">
+        <v>385</v>
+      </c>
+      <c r="E79" t="s">
+        <v>305</v>
+      </c>
+      <c r="F79" t="s">
+        <v>386</v>
+      </c>
+      <c r="G79" t="s">
+        <v>387</v>
+      </c>
+      <c r="H79" t="s">
+        <v>23</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>389</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C80" t="s">
+        <v>374</v>
+      </c>
+      <c r="D80" t="s">
+        <v>390</v>
+      </c>
+      <c r="E80" t="s">
+        <v>391</v>
+      </c>
+      <c r="F80" t="s">
+        <v>392</v>
+      </c>
+      <c r="G80" t="s">
+        <v>393</v>
+      </c>
+      <c r="H80" t="s">
+        <v>23</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>395</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C81" t="s">
+        <v>368</v>
+      </c>
+      <c r="D81" t="s">
+        <v>396</v>
+      </c>
+      <c r="E81" t="s">
+        <v>397</v>
+      </c>
+      <c r="F81" t="s">
+        <v>398</v>
+      </c>
+      <c r="G81" t="s">
+        <v>399</v>
+      </c>
+      <c r="H81" t="s">
+        <v>23</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>401</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C82" t="s">
+        <v>368</v>
+      </c>
+      <c r="D82" t="s">
+        <v>402</v>
+      </c>
+      <c r="E82" t="s">
+        <v>329</v>
+      </c>
+      <c r="F82" t="s">
+        <v>403</v>
+      </c>
+      <c r="G82" t="s">
+        <v>331</v>
+      </c>
+      <c r="H82" t="s">
+        <v>23</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>405</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C83" t="s">
+        <v>368</v>
+      </c>
+      <c r="D83" t="s">
+        <v>406</v>
+      </c>
+      <c r="E83" t="s">
+        <v>407</v>
+      </c>
+      <c r="F83" t="s">
+        <v>408</v>
+      </c>
+      <c r="G83" t="s">
+        <v>409</v>
+      </c>
+      <c r="H83" t="s">
+        <v>23</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>410</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C84" t="s">
+        <v>374</v>
+      </c>
+      <c r="D84" t="s">
+        <v>411</v>
+      </c>
+      <c r="E84" t="s">
+        <v>412</v>
+      </c>
+      <c r="F84" t="s">
+        <v>413</v>
+      </c>
+      <c r="G84" t="s">
+        <v>325</v>
+      </c>
+      <c r="H84" t="s">
+        <v>23</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>415</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C85" t="s">
+        <v>374</v>
+      </c>
+      <c r="D85" t="s">
+        <v>416</v>
+      </c>
+      <c r="E85" t="s">
+        <v>417</v>
+      </c>
+      <c r="F85" t="s">
+        <v>418</v>
+      </c>
+      <c r="G85" t="s">
+        <v>419</v>
+      </c>
+      <c r="H85" t="s">
+        <v>23</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>421</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C86" t="s">
+        <v>368</v>
+      </c>
+      <c r="D86" t="s">
+        <v>422</v>
+      </c>
+      <c r="E86" t="s">
+        <v>347</v>
+      </c>
+      <c r="F86" t="s">
+        <v>423</v>
+      </c>
+      <c r="G86" t="s">
+        <v>424</v>
+      </c>
+      <c r="H86" t="s">
+        <v>23</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>425</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C87" t="s">
+        <v>368</v>
+      </c>
+      <c r="D87" t="s">
+        <v>426</v>
+      </c>
+      <c r="E87" t="s">
+        <v>341</v>
+      </c>
+      <c r="F87" t="s">
+        <v>427</v>
+      </c>
+      <c r="G87" t="s">
+        <v>428</v>
+      </c>
+      <c r="H87" t="s">
+        <v>23</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>429</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C88" t="s">
+        <v>430</v>
+      </c>
+      <c r="D88" t="s">
+        <v>431</v>
+      </c>
+      <c r="E88" t="s">
+        <v>432</v>
+      </c>
+      <c r="F88" t="s">
+        <v>433</v>
+      </c>
+      <c r="G88" t="s">
+        <v>434</v>
+      </c>
+      <c r="H88" t="s">
+        <v>23</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>436</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C89" t="s">
+        <v>430</v>
+      </c>
+      <c r="D89" t="s">
+        <v>437</v>
+      </c>
+      <c r="E89" t="s">
+        <v>438</v>
+      </c>
+      <c r="F89" t="s">
+        <v>439</v>
+      </c>
+      <c r="G89" t="s">
+        <v>440</v>
+      </c>
+      <c r="H89" t="s">
+        <v>23</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>442</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C90" t="s">
+        <v>368</v>
+      </c>
+      <c r="D90" t="s">
+        <v>369</v>
+      </c>
+      <c r="E90" t="s">
+        <v>286</v>
+      </c>
+      <c r="F90" t="s">
+        <v>443</v>
+      </c>
+      <c r="G90" t="s">
+        <v>371</v>
+      </c>
+      <c r="H90" t="s">
+        <v>23</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>445</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C91" t="s">
+        <v>374</v>
+      </c>
+      <c r="D91" t="s">
+        <v>375</v>
+      </c>
+      <c r="E91" t="s">
+        <v>293</v>
+      </c>
+      <c r="F91" t="s">
+        <v>446</v>
+      </c>
+      <c r="G91" t="s">
+        <v>377</v>
+      </c>
+      <c r="H91" t="s">
+        <v>23</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>448</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C92" t="s">
+        <v>374</v>
+      </c>
+      <c r="D92" t="s">
+        <v>380</v>
+      </c>
+      <c r="E92" t="s">
+        <v>299</v>
+      </c>
+      <c r="F92" t="s">
+        <v>449</v>
+      </c>
+      <c r="G92" t="s">
+        <v>382</v>
+      </c>
+      <c r="H92" t="s">
+        <v>23</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>451</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C93" t="s">
+        <v>374</v>
+      </c>
+      <c r="D93" t="s">
+        <v>385</v>
+      </c>
+      <c r="E93" t="s">
+        <v>305</v>
+      </c>
+      <c r="F93" t="s">
+        <v>452</v>
+      </c>
+      <c r="G93" t="s">
+        <v>387</v>
+      </c>
+      <c r="H93" t="s">
+        <v>23</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>454</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C94" t="s">
+        <v>374</v>
+      </c>
+      <c r="D94" t="s">
+        <v>390</v>
+      </c>
+      <c r="E94" t="s">
+        <v>391</v>
+      </c>
+      <c r="F94" t="s">
+        <v>455</v>
+      </c>
+      <c r="G94" t="s">
+        <v>393</v>
+      </c>
+      <c r="H94" t="s">
+        <v>23</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>457</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C95" t="s">
+        <v>368</v>
+      </c>
+      <c r="D95" t="s">
+        <v>396</v>
+      </c>
+      <c r="E95" t="s">
+        <v>458</v>
+      </c>
+      <c r="F95" t="s">
+        <v>459</v>
+      </c>
+      <c r="G95" t="s">
+        <v>399</v>
+      </c>
+      <c r="H95" t="s">
+        <v>23</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>461</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C96" t="s">
+        <v>368</v>
+      </c>
+      <c r="D96" t="s">
+        <v>402</v>
+      </c>
+      <c r="E96" t="s">
+        <v>329</v>
+      </c>
+      <c r="F96" t="s">
+        <v>462</v>
+      </c>
+      <c r="G96" t="s">
+        <v>331</v>
+      </c>
+      <c r="H96" t="s">
+        <v>23</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>464</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C97" t="s">
+        <v>368</v>
+      </c>
+      <c r="D97" t="s">
+        <v>406</v>
+      </c>
+      <c r="E97" t="s">
+        <v>465</v>
+      </c>
+      <c r="F97" t="s">
+        <v>466</v>
+      </c>
+      <c r="G97" t="s">
+        <v>409</v>
+      </c>
+      <c r="H97" t="s">
+        <v>23</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>467</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C98" t="s">
+        <v>374</v>
+      </c>
+      <c r="D98" t="s">
+        <v>411</v>
+      </c>
+      <c r="E98" t="s">
+        <v>468</v>
+      </c>
+      <c r="F98" t="s">
+        <v>469</v>
+      </c>
+      <c r="G98" t="s">
+        <v>325</v>
+      </c>
+      <c r="H98" t="s">
+        <v>23</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>470</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C99" t="s">
+        <v>374</v>
+      </c>
+      <c r="D99" t="s">
+        <v>416</v>
+      </c>
+      <c r="E99" t="s">
+        <v>471</v>
+      </c>
+      <c r="F99" t="s">
+        <v>472</v>
+      </c>
+      <c r="G99" t="s">
+        <v>419</v>
+      </c>
+      <c r="H99" t="s">
+        <v>23</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>474</v>
+      </c>
+      <c r="B100" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C100" t="s">
+        <v>368</v>
+      </c>
+      <c r="D100" t="s">
+        <v>422</v>
+      </c>
+      <c r="E100" t="s">
+        <v>347</v>
+      </c>
+      <c r="F100" t="s">
+        <v>475</v>
+      </c>
+      <c r="G100" t="s">
+        <v>424</v>
+      </c>
+      <c r="H100" t="s">
+        <v>23</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>476</v>
+      </c>
+      <c r="B101" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C101" t="s">
+        <v>368</v>
+      </c>
+      <c r="D101" t="s">
+        <v>426</v>
+      </c>
+      <c r="E101" t="s">
+        <v>341</v>
+      </c>
+      <c r="F101" t="s">
+        <v>477</v>
+      </c>
+      <c r="G101" t="s">
+        <v>428</v>
+      </c>
+      <c r="H101" t="s">
+        <v>23</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>478</v>
+      </c>
+      <c r="B102" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C102" t="s">
+        <v>430</v>
+      </c>
+      <c r="D102" t="s">
+        <v>431</v>
+      </c>
+      <c r="E102" t="s">
+        <v>479</v>
+      </c>
+      <c r="F102" t="s">
+        <v>480</v>
+      </c>
+      <c r="G102" t="s">
+        <v>434</v>
+      </c>
+      <c r="H102" t="s">
+        <v>23</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>482</v>
+      </c>
+      <c r="B103" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C103" t="s">
+        <v>430</v>
+      </c>
+      <c r="D103" t="s">
+        <v>437</v>
+      </c>
+      <c r="E103" t="s">
+        <v>483</v>
+      </c>
+      <c r="F103" t="s">
+        <v>484</v>
+      </c>
+      <c r="G103" t="s">
+        <v>440</v>
+      </c>
+      <c r="H103" t="s">
+        <v>23</v>
+      </c>
+      <c r="I103" s="1" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>486</v>
+      </c>
+      <c r="B104" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="C104" t="s">
+        <v>284</v>
+      </c>
+      <c r="D104" t="s">
+        <v>487</v>
+      </c>
+      <c r="E104" t="s">
+        <v>488</v>
+      </c>
+      <c r="F104" t="s">
+        <v>489</v>
+      </c>
+      <c r="G104" t="s">
+        <v>490</v>
+      </c>
+      <c r="H104" t="s">
+        <v>23</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>491</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>